<commit_message>
Added Montserrat, basic styling started
</commit_message>
<xml_diff>
--- a/time-spent.xlsx
+++ b/time-spent.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\smccann-software\smwebman\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A622B06-35C4-491A-96F5-7BF4D7C43D5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63102A29-E3E5-4EE7-9A98-0CA5D555E4E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{A10B42A8-E862-4DE3-8908-170894873712}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="7">
   <si>
     <t>Content and basic structure</t>
   </si>
@@ -54,6 +54,9 @@
   </si>
   <si>
     <t>Tasks</t>
+  </si>
+  <si>
+    <t>Logo</t>
   </si>
 </sst>
 </file>
@@ -437,7 +440,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CEDC7E68-DEF6-4655-B185-A65A633E6874}">
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -469,7 +472,7 @@
       </c>
       <c r="M1" s="4">
         <f>SUM(D:D)</f>
-        <v>3.6111111111111094E-2</v>
+        <v>0.27569444444444441</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
@@ -505,6 +508,84 @@
         <v>1.388888888888884E-2</v>
       </c>
       <c r="F3" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A4" s="1">
+        <v>45878</v>
+      </c>
+      <c r="B4" s="2">
+        <v>0.39583333333333331</v>
+      </c>
+      <c r="C4" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="D4" s="2">
+        <f t="shared" ref="D4:D10" si="0">C4-B4</f>
+        <v>0.10416666666666669</v>
+      </c>
+      <c r="F4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A5" s="1">
+        <v>45879</v>
+      </c>
+      <c r="B5" s="2">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="C5" s="2">
+        <v>0.47916666666666669</v>
+      </c>
+      <c r="D5" s="2">
+        <f t="shared" si="0"/>
+        <v>6.25E-2</v>
+      </c>
+      <c r="F5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A6" s="1">
+        <v>45879</v>
+      </c>
+      <c r="B6" s="2">
+        <v>0.70833333333333337</v>
+      </c>
+      <c r="C6" s="2">
+        <v>0.78125</v>
+      </c>
+      <c r="D6" s="2">
+        <f t="shared" si="0"/>
+        <v>7.291666666666663E-2</v>
+      </c>
+      <c r="F6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="D7" s="2">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="D8" s="2">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="D9" s="2">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="D10" s="2">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>

</xml_diff>